<commit_message>
fix: ecuacion Hatch no-lineal completa (brentq) + heat_capacity_ratio + dispersividad beta
Corrige 3 bugs criticos en _flux_hatch_amplitude:
1. Ecuacion simplificada -> Hatch (2006) Eq.6a completa con brentq
2. Agrega heat_capacity_ratio (Cs/Cw) para convertir v_thermal -> seepage flux
3. Agrega dispersividad termica beta (d50) en difusividad efectiva

Resultados ANTES vs DESPUES (ajuste global):
  TC1: 133 -> 337 mm/d (MATLAB 281, delta +20%)
  TC2:  55 -> 316 mm/d (MATLAB 311, delta +1.6%)
  TC3:  10 -> 664 mm/d (MATLAB 2246, delta -70%)
  TC4:  26 -> 678 mm/d (MATLAB 1555, delta -56%)
  TC5: 213 -> 220 mm/d (MATLAB 181, delta +22%)

TC3/TC4 discrepancia residual por DHR vs ajuste global.
Series temporales ventana deslizante muestran TC3/TC4 dentro del rango MATLAB.
</commit_message>
<xml_diff>
--- a/resultados_python/terreno_2026_hatch/resultados_05A_hatch_amplitude.xlsx
+++ b/resultados_python/terreno_2026_hatch/resultados_05A_hatch_amplitude.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="Flujos_HA_McCallum" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Flujo_Promedio_TC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Confiabilidad" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Incertidumbre" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Analisis_Armonico" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Params_IDIEM" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="IQR_Hatch_Amplitude" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Confiabilidad" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Incertidumbre" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Analisis_Armonico" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Params_IDIEM" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,10 +471,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>143.87</v>
+        <v>319.11</v>
       </c>
       <c r="E2" t="n">
-        <v>1.665163826138439e-06</v>
+        <v>3.693410180727508e-06</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -526,10 +527,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>122.66</v>
+        <v>355.84</v>
       </c>
       <c r="E4" t="n">
-        <v>1.41961856650084e-06</v>
+        <v>4.118472100721804e-06</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -582,10 +583,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>133.26</v>
+        <v>336.86</v>
       </c>
       <c r="E6" t="n">
-        <v>1.54239119631964e-06</v>
+        <v>3.898873925546228e-06</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -638,10 +639,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>51.17</v>
+        <v>328.48</v>
       </c>
       <c r="E8" t="n">
-        <v>5.922032834209716e-07</v>
+        <v>3.801852538530034e-06</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -694,10 +695,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>58.63</v>
+        <v>303.68</v>
       </c>
       <c r="E10" t="n">
-        <v>6.786256664778579e-07</v>
+        <v>3.51479590257698e-06</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -750,10 +751,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>54.9</v>
+        <v>315.69</v>
       </c>
       <c r="E12" t="n">
-        <v>6.354144749494147e-07</v>
+        <v>3.65383361088845e-06</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -806,10 +807,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13.83</v>
+        <v>570.91</v>
       </c>
       <c r="E14" t="n">
-        <v>1.600278250125927e-07</v>
+        <v>6.607727801064487e-06</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -862,10 +863,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5.79</v>
+        <v>775.5700000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>6.696753633364922e-08</v>
+        <v>8.976545513397485e-06</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -918,10 +919,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9.81</v>
+        <v>645.7</v>
       </c>
       <c r="E18" t="n">
-        <v>1.13497680673121e-07</v>
+        <v>7.473382200419429e-06</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -974,10 +975,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>28.23</v>
+        <v>654.04</v>
       </c>
       <c r="E20" t="n">
-        <v>3.266834961863177e-07</v>
+        <v>7.569899553840944e-06</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1030,10 +1031,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>23.09</v>
+        <v>702.58</v>
       </c>
       <c r="E22" t="n">
-        <v>2.672973344789684e-07</v>
+        <v>8.131685023806157e-06</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1086,10 +1087,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>25.66</v>
+        <v>676.77</v>
       </c>
       <c r="E24" t="n">
-        <v>2.969904153326433e-07</v>
+        <v>7.832967858553909e-06</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1142,10 +1143,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>296.4</v>
+        <v>135.1</v>
       </c>
       <c r="E26" t="n">
-        <v>3.430526789539439e-06</v>
+        <v>1.563618403454325e-06</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1198,10 +1199,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>129.2</v>
+        <v>314.12</v>
       </c>
       <c r="E28" t="n">
-        <v>1.495391369014579e-06</v>
+        <v>3.635606922535975e-06</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1254,10 +1255,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>212.8</v>
+        <v>211.78</v>
       </c>
       <c r="E30" t="n">
-        <v>2.462959079277009e-06</v>
+        <v>2.451183073645845e-06</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1366,10 +1367,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>133.26</v>
+        <v>337.27</v>
       </c>
       <c r="C2" t="n">
-        <v>10.61</v>
+        <v>18.37</v>
       </c>
       <c r="D2" t="n">
         <v>484.47</v>
@@ -1402,10 +1403,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54.9</v>
+        <v>315.95</v>
       </c>
       <c r="C3" t="n">
-        <v>3.73</v>
+        <v>12.4</v>
       </c>
       <c r="D3" t="n">
         <v>297.25</v>
@@ -1438,10 +1439,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.81</v>
+        <v>664.0599999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>4.02</v>
+        <v>103.56</v>
       </c>
       <c r="D4" t="n">
         <v>40.65</v>
@@ -1474,10 +1475,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25.66</v>
+        <v>677.8</v>
       </c>
       <c r="C5" t="n">
-        <v>2.57</v>
+        <v>24.29</v>
       </c>
       <c r="D5" t="n">
         <v>76.67</v>
@@ -1510,10 +1511,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>212.8</v>
+        <v>220.33</v>
       </c>
       <c r="C6" t="n">
-        <v>83.59999999999999</v>
+        <v>89.81999999999999</v>
       </c>
       <c r="D6" t="n">
         <v>1212.83</v>
@@ -1550,7 +1551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1561,47 +1562,42 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Par</t>
+          <t>HA_medio_mm_d</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>IC_total</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>R2_sup</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>R2_inf</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Concord_HA_MC</t>
+          <t>Desv_Est</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>IC_lit</t>
+          <t>n_pares</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>IC_physics</t>
+          <t>MATLAB_ref_mm_d</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>HA_mm_d</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>MC_mm_d</t>
+          <t>Delta_pct</t>
         </is>
       </c>
     </row>
@@ -1611,538 +1607,153 @@
           <t>TC1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>sup→int</t>
-        </is>
+      <c r="B2" t="n">
+        <v>337.3</v>
       </c>
       <c r="C2" t="n">
-        <v>0.709</v>
+        <v>328</v>
       </c>
       <c r="D2" t="n">
-        <v>0.728</v>
+        <v>336.9</v>
       </c>
       <c r="E2" t="n">
-        <v>0.483</v>
+        <v>346.3</v>
       </c>
       <c r="F2" t="n">
-        <v>0.522</v>
+        <v>18.4</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>281</v>
       </c>
       <c r="I2" t="n">
-        <v>143.9</v>
-      </c>
-      <c r="J2" t="n">
-        <v>275.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TC1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>int→inf</t>
-        </is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>315.9</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6</v>
+        <v>309.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.483</v>
+        <v>315.7</v>
       </c>
       <c r="E3" t="n">
-        <v>0.103</v>
+        <v>322.1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.635</v>
+        <v>12.4</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>311</v>
       </c>
       <c r="I3" t="n">
-        <v>122.7</v>
-      </c>
-      <c r="J3" t="n">
-        <v>193.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>sup→inf</t>
-        </is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>664.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.536</v>
+        <v>608.3</v>
       </c>
       <c r="D4" t="n">
-        <v>0.728</v>
+        <v>645.7</v>
       </c>
       <c r="E4" t="n">
-        <v>0.103</v>
+        <v>710.6</v>
       </c>
       <c r="F4" t="n">
-        <v>0.135</v>
+        <v>103.6</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2246</v>
       </c>
       <c r="I4" t="n">
-        <v>133.3</v>
-      </c>
-      <c r="J4" t="n">
-        <v>984.7</v>
+        <v>-70.40000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>sup→int</t>
-        </is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>677.8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6</v>
+        <v>665.4</v>
       </c>
       <c r="D5" t="n">
-        <v>0.619</v>
+        <v>676.8</v>
       </c>
       <c r="E5" t="n">
-        <v>0.218</v>
+        <v>689.7</v>
       </c>
       <c r="F5" t="n">
-        <v>0.408</v>
+        <v>24.3</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>1555</v>
       </c>
       <c r="I5" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="J5" t="n">
-        <v>125.4</v>
+        <v>-56.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TC2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>int→inf</t>
-        </is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>220.3</v>
       </c>
       <c r="C6" t="n">
-        <v>0.465</v>
+        <v>173.4</v>
       </c>
       <c r="D6" t="n">
-        <v>0.218</v>
+        <v>211.8</v>
       </c>
       <c r="E6" t="n">
-        <v>0.022</v>
+        <v>262.9</v>
       </c>
       <c r="F6" t="n">
-        <v>0.425</v>
+        <v>89.8</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>181</v>
       </c>
       <c r="I6" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="J6" t="n">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TC2</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>sup→inf</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.619</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="J7" t="n">
-        <v>628.3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sup→int</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.722</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.606</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.496</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="J8" t="n">
-        <v>27.9</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>int→inf</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.6879999999999999</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.6919999999999999</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.523</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="J9" t="n">
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>sup→inf</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.617</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.606</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.6919999999999999</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.118</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="J10" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>sup→int</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.836</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.782</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="n">
-        <v>28.2</v>
-      </c>
-      <c r="J11" t="n">
-        <v>41.7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>int→inf</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0.8179999999999999</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.782</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.6889999999999999</v>
-      </c>
-      <c r="G12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="J12" t="n">
-        <v>33.5</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>sup→inf</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.836</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.166</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="J13" t="n">
-        <v>154.7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>sup→int</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>0.634</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.422</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" t="n">
-        <v>296.4</v>
-      </c>
-      <c r="J14" t="n">
-        <v>703</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>int→inf</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>0.428</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.368</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="n">
-        <v>129.2</v>
-      </c>
-      <c r="J15" t="n">
-        <v>351.3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>sup→inf</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0.528</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="G16" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="n">
-        <v>212.8</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2584.2</v>
+        <v>21.7</v>
       </c>
     </row>
   </sheetData>
@@ -2156,7 +1767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2172,32 +1783,42 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Flujo HA (mm/d)</t>
+          <t>IC_total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>u_rel (%)</t>
+          <t>R2_sup</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>u_abs (mm/d)</t>
+          <t>R2_inf</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>IC 95% bajo</t>
+          <t>Concord_HA_MC</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>IC 95% alto</t>
+          <t>IC_lit</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>u_armónico (%)</t>
+          <t>IC_physics</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>HA_mm_d</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>MC_mm_d</t>
         </is>
       </c>
     </row>
@@ -2213,22 +1834,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>143.9</v>
+        <v>0.795</v>
       </c>
       <c r="D2" t="n">
-        <v>12.9</v>
+        <v>0.728</v>
       </c>
       <c r="E2" t="n">
-        <v>18.6</v>
+        <v>0.483</v>
       </c>
       <c r="F2" t="n">
-        <v>107.4</v>
+        <v>0.864</v>
       </c>
       <c r="G2" t="n">
-        <v>180.3</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>319.1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>275.7</v>
       </c>
     </row>
     <row r="3">
@@ -2243,22 +1870,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>122.7</v>
+        <v>0.577</v>
       </c>
       <c r="D3" t="n">
-        <v>21.6</v>
+        <v>0.483</v>
       </c>
       <c r="E3" t="n">
-        <v>26.5</v>
+        <v>0.103</v>
       </c>
       <c r="F3" t="n">
-        <v>70.7</v>
+        <v>0.543</v>
       </c>
       <c r="G3" t="n">
-        <v>174.6</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>355.8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>193.1</v>
       </c>
     </row>
     <row r="4">
@@ -2273,22 +1906,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>133.3</v>
+        <v>0.588</v>
       </c>
       <c r="D4" t="n">
-        <v>21.6</v>
+        <v>0.728</v>
       </c>
       <c r="E4" t="n">
-        <v>28.8</v>
+        <v>0.103</v>
       </c>
       <c r="F4" t="n">
-        <v>76.8</v>
+        <v>0.342</v>
       </c>
       <c r="G4" t="n">
-        <v>189.7</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>336.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>984.7</v>
       </c>
     </row>
     <row r="5">
@@ -2303,22 +1942,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51.2</v>
+        <v>0.594</v>
       </c>
       <c r="D5" t="n">
-        <v>21.6</v>
+        <v>0.619</v>
       </c>
       <c r="E5" t="n">
-        <v>11.1</v>
+        <v>0.218</v>
       </c>
       <c r="F5" t="n">
-        <v>29.5</v>
+        <v>0.382</v>
       </c>
       <c r="G5" t="n">
-        <v>72.8</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>328.5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>125.4</v>
       </c>
     </row>
     <row r="6">
@@ -2333,22 +1978,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>58.6</v>
+        <v>0.472</v>
       </c>
       <c r="D6" t="n">
-        <v>21.6</v>
+        <v>0.218</v>
       </c>
       <c r="E6" t="n">
-        <v>12.7</v>
+        <v>0.022</v>
       </c>
       <c r="F6" t="n">
-        <v>33.8</v>
+        <v>0.454</v>
       </c>
       <c r="G6" t="n">
-        <v>83.5</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>303.7</v>
+      </c>
+      <c r="J6" t="n">
+        <v>138</v>
       </c>
     </row>
     <row r="7">
@@ -2363,22 +2014,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>54.9</v>
+        <v>0.585</v>
       </c>
       <c r="D7" t="n">
-        <v>21.6</v>
+        <v>0.619</v>
       </c>
       <c r="E7" t="n">
-        <v>11.9</v>
+        <v>0.022</v>
       </c>
       <c r="F7" t="n">
-        <v>31.6</v>
+        <v>0.502</v>
       </c>
       <c r="G7" t="n">
-        <v>78.2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>315.7</v>
+      </c>
+      <c r="J7" t="n">
+        <v>628.3</v>
       </c>
     </row>
     <row r="8">
@@ -2393,22 +2050,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13.8</v>
+        <v>0.61</v>
       </c>
       <c r="D8" t="n">
-        <v>12.9</v>
+        <v>0.606</v>
       </c>
       <c r="E8" t="n">
-        <v>1.8</v>
+        <v>0.73</v>
       </c>
       <c r="F8" t="n">
-        <v>10.3</v>
+        <v>0.049</v>
       </c>
       <c r="G8" t="n">
-        <v>17.3</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>570.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>27.9</v>
       </c>
     </row>
     <row r="9">
@@ -2423,22 +2086,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5.8</v>
+        <v>0.581</v>
       </c>
       <c r="D9" t="n">
-        <v>12.9</v>
+        <v>0.73</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>4.3</v>
+        <v>0.014</v>
       </c>
       <c r="G9" t="n">
-        <v>7.3</v>
+        <v>0.707</v>
       </c>
       <c r="H9" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>775.6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>11.1</v>
       </c>
     </row>
     <row r="10">
@@ -2453,22 +2122,28 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9.800000000000001</v>
+        <v>0.611</v>
       </c>
       <c r="D10" t="n">
-        <v>12.9</v>
+        <v>0.606</v>
       </c>
       <c r="E10" t="n">
-        <v>1.3</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>7.3</v>
+        <v>0.129</v>
       </c>
       <c r="G10" t="n">
-        <v>12.3</v>
+        <v>0.924</v>
       </c>
       <c r="H10" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>645.7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="11">
@@ -2483,22 +2158,28 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28.2</v>
+        <v>0.668</v>
       </c>
       <c r="D11" t="n">
-        <v>9.6</v>
+        <v>0.836</v>
       </c>
       <c r="E11" t="n">
-        <v>2.7</v>
+        <v>0.782</v>
       </c>
       <c r="F11" t="n">
-        <v>22.9</v>
+        <v>0.064</v>
       </c>
       <c r="G11" t="n">
-        <v>33.5</v>
+        <v>0.91</v>
       </c>
       <c r="H11" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>654</v>
+      </c>
+      <c r="J11" t="n">
+        <v>41.7</v>
       </c>
     </row>
     <row r="12">
@@ -2513,22 +2194,28 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>23.1</v>
+        <v>0.632</v>
       </c>
       <c r="D12" t="n">
-        <v>12.9</v>
+        <v>0.782</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>0.75</v>
       </c>
       <c r="F12" t="n">
-        <v>17.2</v>
+        <v>0.048</v>
       </c>
       <c r="G12" t="n">
-        <v>28.9</v>
+        <v>0.829</v>
       </c>
       <c r="H12" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>702.6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>33.5</v>
       </c>
     </row>
     <row r="13">
@@ -2543,22 +2230,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>25.7</v>
+        <v>0.697</v>
       </c>
       <c r="D13" t="n">
-        <v>12.9</v>
+        <v>0.836</v>
       </c>
       <c r="E13" t="n">
-        <v>3.3</v>
+        <v>0.75</v>
       </c>
       <c r="F13" t="n">
-        <v>19.2</v>
+        <v>0.229</v>
       </c>
       <c r="G13" t="n">
-        <v>32.2</v>
+        <v>0.872</v>
       </c>
       <c r="H13" t="n">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>676.8</v>
+      </c>
+      <c r="J13" t="n">
+        <v>154.7</v>
       </c>
     </row>
     <row r="14">
@@ -2573,22 +2266,28 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>296.4</v>
+        <v>0.577</v>
       </c>
       <c r="D14" t="n">
-        <v>21.6</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>64.09999999999999</v>
+        <v>0.128</v>
       </c>
       <c r="F14" t="n">
-        <v>170.8</v>
+        <v>0.192</v>
       </c>
       <c r="G14" t="n">
-        <v>422</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>135.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>703</v>
       </c>
     </row>
     <row r="15">
@@ -2603,22 +2302,28 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>129.2</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>21.6</v>
+        <v>0.128</v>
       </c>
       <c r="E15" t="n">
-        <v>27.9</v>
+        <v>0.023</v>
       </c>
       <c r="F15" t="n">
-        <v>74.5</v>
+        <v>0.894</v>
       </c>
       <c r="G15" t="n">
-        <v>183.9</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>314.1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>351.3</v>
       </c>
     </row>
     <row r="16">
@@ -2633,22 +2338,28 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>212.8</v>
+        <v>0.528</v>
       </c>
       <c r="D16" t="n">
-        <v>21.6</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>46</v>
+        <v>0.023</v>
       </c>
       <c r="F16" t="n">
-        <v>122.6</v>
+        <v>0.082</v>
       </c>
       <c r="G16" t="n">
-        <v>303</v>
+        <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>211.8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2584.2</v>
       </c>
     </row>
   </sheetData>
@@ -2662,549 +2373,499 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sensor</t>
+          <t>TC</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>Par</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>profundidad_m</t>
+          <t>Flujo HA (mm/d)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>amplitud_C</t>
+          <t>u_rel (%)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>fase_rad</t>
+          <t>u_abs (mm/d)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>fase_deg</t>
+          <t>IC 95% bajo</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>offset_C</t>
+          <t>IC 95% alto</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>n_dias_ajuste</t>
+          <t>u_armónico (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>temp_12</t>
+          <t>TC1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>sup→int</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>319.1</v>
       </c>
       <c r="D2" t="n">
-        <v>5.152</v>
+        <v>12.9</v>
       </c>
       <c r="E2" t="n">
-        <v>1.5242</v>
+        <v>41.3</v>
       </c>
       <c r="F2" t="n">
-        <v>87.3</v>
+        <v>238.2</v>
       </c>
       <c r="G2" t="n">
-        <v>18.28</v>
+        <v>400</v>
       </c>
       <c r="H2" t="n">
-        <v>0.728</v>
-      </c>
-      <c r="I2" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>temp_9</t>
+          <t>TC1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>int→inf</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.28</v>
+        <v>355.8</v>
       </c>
       <c r="D3" t="n">
-        <v>1.4228</v>
+        <v>21.6</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1391</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>205.1</v>
       </c>
       <c r="G3" t="n">
-        <v>17.49</v>
+        <v>506.6</v>
       </c>
       <c r="H3" t="n">
-        <v>0.483</v>
-      </c>
-      <c r="I3" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>temp_8</t>
+          <t>TC1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>sup→inf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5600000000000001</v>
+        <v>336.9</v>
       </c>
       <c r="D4" t="n">
-        <v>0.475</v>
+        <v>21.6</v>
       </c>
       <c r="E4" t="n">
-        <v>6.2051</v>
+        <v>72.8</v>
       </c>
       <c r="F4" t="n">
-        <v>355.5</v>
+        <v>194.2</v>
       </c>
       <c r="G4" t="n">
-        <v>17.57</v>
+        <v>479.6</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1028</v>
-      </c>
-      <c r="I4" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>temp_4</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>sup→int</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>328.5</v>
       </c>
       <c r="D5" t="n">
-        <v>2.4911</v>
+        <v>21.6</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3039</v>
+        <v>71</v>
       </c>
       <c r="F5" t="n">
-        <v>17.4</v>
+        <v>189.3</v>
       </c>
       <c r="G5" t="n">
-        <v>17.01</v>
+        <v>467.6</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6192</v>
-      </c>
-      <c r="I5" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>temp_6</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>int→inf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.2</v>
+        <v>303.7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7324000000000001</v>
+        <v>21.6</v>
       </c>
       <c r="E6" t="n">
-        <v>4.9513</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>283.7</v>
+        <v>175</v>
       </c>
       <c r="G6" t="n">
-        <v>17.15</v>
+        <v>432.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.218</v>
-      </c>
-      <c r="I6" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>temp_7</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>sup→inf</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.4</v>
+        <v>315.7</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1801</v>
+        <v>21.6</v>
       </c>
       <c r="E7" t="n">
-        <v>3.4749</v>
+        <v>68.2</v>
       </c>
       <c r="F7" t="n">
-        <v>199.1</v>
+        <v>182</v>
       </c>
       <c r="G7" t="n">
-        <v>17.3</v>
+        <v>449.4</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0216</v>
-      </c>
-      <c r="I7" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>temp_1</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>sup→int</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>570.9</v>
       </c>
       <c r="D8" t="n">
-        <v>5.0217</v>
+        <v>12.9</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4528</v>
+        <v>73.8</v>
       </c>
       <c r="F8" t="n">
-        <v>25.9</v>
+        <v>426.2</v>
       </c>
       <c r="G8" t="n">
-        <v>18.4</v>
+        <v>715.6</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6062</v>
-      </c>
-      <c r="I8" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>temp_10</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>int→inf</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.2</v>
+        <v>775.6</v>
       </c>
       <c r="D9" t="n">
-        <v>3.7429</v>
+        <v>12.9</v>
       </c>
       <c r="E9" t="n">
-        <v>6.1382</v>
+        <v>100.3</v>
       </c>
       <c r="F9" t="n">
-        <v>351.7</v>
+        <v>579</v>
       </c>
       <c r="G9" t="n">
-        <v>18.07</v>
+        <v>972.1</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7295</v>
-      </c>
-      <c r="I9" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>temp_11</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>sup→inf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.4</v>
+        <v>645.7</v>
       </c>
       <c r="D10" t="n">
-        <v>3.3097</v>
+        <v>12.9</v>
       </c>
       <c r="E10" t="n">
-        <v>5.8559</v>
+        <v>83.5</v>
       </c>
       <c r="F10" t="n">
-        <v>335.5</v>
+        <v>482.1</v>
       </c>
       <c r="G10" t="n">
-        <v>18.09</v>
+        <v>809.3</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6924</v>
-      </c>
-      <c r="I10" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>temp_15</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TC4</t>
+          <t>sup→int</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>654</v>
       </c>
       <c r="D11" t="n">
-        <v>4.7744</v>
+        <v>9.6</v>
       </c>
       <c r="E11" t="n">
-        <v>1.2132</v>
+        <v>62.8</v>
       </c>
       <c r="F11" t="n">
-        <v>69.5</v>
+        <v>531</v>
       </c>
       <c r="G11" t="n">
-        <v>18.49</v>
+        <v>777.1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.8363</v>
-      </c>
-      <c r="I11" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>temp_3</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TC4</t>
+          <t>int→inf</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.28</v>
+        <v>702.6</v>
       </c>
       <c r="D12" t="n">
-        <v>4.0651</v>
+        <v>12.9</v>
       </c>
       <c r="E12" t="n">
-        <v>0.978</v>
+        <v>90.8</v>
       </c>
       <c r="F12" t="n">
-        <v>56</v>
+        <v>524.5</v>
       </c>
       <c r="G12" t="n">
-        <v>18.25</v>
+        <v>880.6</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7824</v>
-      </c>
-      <c r="I12" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>temp_14</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TC4</t>
+          <t>sup→inf</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.5600000000000001</v>
+        <v>676.8</v>
       </c>
       <c r="D13" t="n">
-        <v>3.5639</v>
+        <v>12.9</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8567</v>
+        <v>87.5</v>
       </c>
       <c r="F13" t="n">
-        <v>49.1</v>
+        <v>505.3</v>
       </c>
       <c r="G13" t="n">
-        <v>18.31</v>
+        <v>848.3</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7496</v>
-      </c>
-      <c r="I13" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>temp_5</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TC5</t>
+          <t>sup→int</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>135.1</v>
       </c>
       <c r="D14" t="n">
-        <v>3.0853</v>
+        <v>21.6</v>
       </c>
       <c r="E14" t="n">
-        <v>1.0866</v>
+        <v>29.2</v>
       </c>
       <c r="F14" t="n">
-        <v>62.3</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>18.23</v>
+        <v>192.3</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8128</v>
-      </c>
-      <c r="I14" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>temp_13</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TC5</t>
+          <t>int→inf</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.28</v>
+        <v>314.1</v>
       </c>
       <c r="D15" t="n">
-        <v>0.33</v>
+        <v>21.6</v>
       </c>
       <c r="E15" t="n">
-        <v>4.8139</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>275.8</v>
+        <v>181</v>
       </c>
       <c r="G15" t="n">
-        <v>18.33</v>
+        <v>447.2</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1276</v>
-      </c>
-      <c r="I15" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>temp_2</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TC5</t>
+          <t>sup→inf</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.5600000000000001</v>
+        <v>211.8</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1246</v>
+        <v>21.6</v>
       </c>
       <c r="E16" t="n">
-        <v>2.1943</v>
+        <v>45.8</v>
       </c>
       <c r="F16" t="n">
-        <v>125.7</v>
+        <v>122.1</v>
       </c>
       <c r="G16" t="n">
-        <v>18.2</v>
+        <v>301.5</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="I16" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -3218,6 +2879,562 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sensor</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>profundidad_m</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>amplitud_C</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fase_rad</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fase_deg</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>offset_C</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>n_dias_ajuste</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>temp_12</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.152</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.5242</v>
+      </c>
+      <c r="F2" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>18.28</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="I2" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>temp_9</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.4228</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1391</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="I3" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>temp_8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6.2051</v>
+      </c>
+      <c r="F4" t="n">
+        <v>355.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>17.57</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1028</v>
+      </c>
+      <c r="I4" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>temp_4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.4911</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3039</v>
+      </c>
+      <c r="F5" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.6192</v>
+      </c>
+      <c r="I5" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>temp_6</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.7324000000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.9513</v>
+      </c>
+      <c r="F6" t="n">
+        <v>283.7</v>
+      </c>
+      <c r="G6" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="I6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>temp_7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1801</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3.4749</v>
+      </c>
+      <c r="F7" t="n">
+        <v>199.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0216</v>
+      </c>
+      <c r="I7" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>temp_1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.0217</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.4528</v>
+      </c>
+      <c r="F8" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.6062</v>
+      </c>
+      <c r="I8" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>temp_10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.7429</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.1382</v>
+      </c>
+      <c r="F9" t="n">
+        <v>351.7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>18.07</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.7295</v>
+      </c>
+      <c r="I9" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>temp_11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.3097</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.8559</v>
+      </c>
+      <c r="F10" t="n">
+        <v>335.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.6924</v>
+      </c>
+      <c r="I10" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>temp_15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.7744</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.2132</v>
+      </c>
+      <c r="F11" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18.49</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.8363</v>
+      </c>
+      <c r="I11" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>temp_3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.0651</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="F12" t="n">
+        <v>56</v>
+      </c>
+      <c r="G12" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.7824</v>
+      </c>
+      <c r="I12" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>temp_14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.5639</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.8567</v>
+      </c>
+      <c r="F13" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>18.31</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.7496</v>
+      </c>
+      <c r="I13" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>temp_5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.0853</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.0866</v>
+      </c>
+      <c r="F14" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G14" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.8128</v>
+      </c>
+      <c r="I14" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>temp_13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.8139</v>
+      </c>
+      <c r="F15" t="n">
+        <v>275.8</v>
+      </c>
+      <c r="G15" t="n">
+        <v>18.33</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.1276</v>
+      </c>
+      <c r="I15" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>temp_2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1246</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.1943</v>
+      </c>
+      <c r="F16" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="G16" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="I16" t="n">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
feat: Add stages for time series analysis, reliability metrics, uncertainty propagation, and export functionality
- Implemented stage 5 for calculating time series of flow using sliding windows.
- Added stage 6 to compute reliability metrics (IC) for sensor pairs.
- Introduced stage 7 for quadratic uncertainty propagation based on IDIEM parameters.
- Created stage 8 for exporting results to multi-sheet Excel and individual CSV files.
- Developed stage 9 for generating executive summaries and IQR tables from time series.
- Added stage 10 for generating static figures using matplotlib.
- Implemented stage 11 for creating interactive HTML panels using Plotly and Folium.
</commit_message>
<xml_diff>
--- a/resultados_python/terreno_2026_hatch/resultados_05A_hatch_amplitude.xlsx
+++ b/resultados_python/terreno_2026_hatch/resultados_05A_hatch_amplitude.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,22 +435,22 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Método</t>
+          <t>HA_mm_d</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>q (mm/día)</t>
+          <t>MC_mm_d</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>q (m/s)</t>
+          <t>Ar</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>dz_m</t>
         </is>
       </c>
     </row>
@@ -462,24 +462,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>314.1</v>
       </c>
       <c r="D2" t="n">
-        <v>319.11</v>
+        <v>275.7</v>
       </c>
       <c r="E2" t="n">
-        <v>3.693410180727508e-06</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.2762</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="3">
@@ -490,24 +486,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>381.9</v>
       </c>
       <c r="D3" t="n">
-        <v>275.67</v>
+        <v>193.1</v>
       </c>
       <c r="E3" t="n">
-        <v>3.190570425739345e-06</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.3339</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="4">
@@ -518,780 +510,308 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>345.9</v>
       </c>
       <c r="D4" t="n">
-        <v>355.84</v>
+        <v>984.7</v>
       </c>
       <c r="E4" t="n">
-        <v>4.118472100721804e-06</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.0922</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>345.1</v>
       </c>
       <c r="D5" t="n">
-        <v>193.07</v>
+        <v>125.4</v>
       </c>
       <c r="E5" t="n">
-        <v>2.234638415168245e-06</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.294</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>315.9</v>
       </c>
       <c r="D6" t="n">
-        <v>336.86</v>
+        <v>138</v>
       </c>
       <c r="E6" t="n">
-        <v>3.898873925546228e-06</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.2459</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC1</t>
+          <t>TC2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>330</v>
       </c>
       <c r="D7" t="n">
-        <v>984.6799999999999</v>
+        <v>628.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.139672433518691e-05</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.0723</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1281.9</v>
       </c>
       <c r="D8" t="n">
-        <v>328.48</v>
+        <v>27.9</v>
       </c>
       <c r="E8" t="n">
-        <v>3.801852538530034e-06</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.7453</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2255.6</v>
       </c>
       <c r="D9" t="n">
-        <v>125.44</v>
+        <v>11.1</v>
       </c>
       <c r="E9" t="n">
-        <v>1.451841111504446e-06</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.8843</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1622.7</v>
       </c>
       <c r="D10" t="n">
-        <v>303.68</v>
+        <v>83</v>
       </c>
       <c r="E10" t="n">
-        <v>3.51479590257698e-06</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.6591</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1617.1</v>
       </c>
       <c r="D11" t="n">
-        <v>137.96</v>
+        <v>41.7</v>
       </c>
       <c r="E11" t="n">
-        <v>1.596802631616574e-06</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.8514</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1868.1</v>
       </c>
       <c r="D12" t="n">
-        <v>315.69</v>
+        <v>33.5</v>
       </c>
       <c r="E12" t="n">
-        <v>3.65383361088845e-06</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.8767</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TC2</t>
+          <t>TC4</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1733.5</v>
       </c>
       <c r="D13" t="n">
-        <v>628.34</v>
+        <v>154.7</v>
       </c>
       <c r="E13" t="n">
-        <v>7.272501502787227e-06</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.7465000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>113.7</v>
       </c>
       <c r="D14" t="n">
-        <v>570.91</v>
+        <v>703</v>
       </c>
       <c r="E14" t="n">
-        <v>6.607727801064487e-06</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.107</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>345.6</v>
       </c>
       <c r="D15" t="n">
-        <v>27.86</v>
+        <v>351.3</v>
       </c>
       <c r="E15" t="n">
-        <v>3.224415901201933e-07</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.3774</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TC3</t>
+          <t>TC5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>200.7</v>
       </c>
       <c r="D16" t="n">
-        <v>775.5700000000001</v>
+        <v>2584.2</v>
       </c>
       <c r="E16" t="n">
-        <v>8.976545513397485e-06</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>11.06</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1.279833689090414e-07</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>645.7</v>
-      </c>
-      <c r="E18" t="n">
-        <v>7.473382200419429e-06</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>83.03</v>
-      </c>
-      <c r="E19" t="n">
-        <v>9.609708398570597e-07</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>654.04</v>
-      </c>
-      <c r="E20" t="n">
-        <v>7.569899553840944e-06</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>41.74</v>
-      </c>
-      <c r="E21" t="n">
-        <v>4.830467113183908e-07</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>702.58</v>
-      </c>
-      <c r="E22" t="n">
-        <v>8.131685023806157e-06</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>33.52</v>
-      </c>
-      <c r="E23" t="n">
-        <v>3.879804188369026e-07</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>676.77</v>
-      </c>
-      <c r="E24" t="n">
-        <v>7.832967858553909e-06</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>154.74</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1.790987078277026e-06</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>135.1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>1.563618403454325e-06</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>sup-int</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>702.98</v>
-      </c>
-      <c r="E27" t="n">
-        <v>8.136333216078073e-06</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>314.12</v>
-      </c>
-      <c r="E28" t="n">
-        <v>3.635606922535975e-06</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>int-inf</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>351.31</v>
-      </c>
-      <c r="E29" t="n">
-        <v>4.066099638411199e-06</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Hatch-Amplitude</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>211.78</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2.451183073645845e-06</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>TC5</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>sup-inf</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>McCallum</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>2584.19</v>
-      </c>
-      <c r="E31" t="n">
-        <v>2.99095731723629e-05</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Infiltración ↓</t>
-        </is>
+        <v>0.0404</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.5600000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1367,16 +887,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>337.27</v>
+        <v>347.3</v>
       </c>
       <c r="C2" t="n">
-        <v>18.37</v>
+        <v>33.92</v>
       </c>
       <c r="D2" t="n">
-        <v>484.47</v>
+        <v>484.5</v>
       </c>
       <c r="E2" t="n">
-        <v>435.16</v>
+        <v>435.15</v>
       </c>
       <c r="F2" t="n">
         <v>0.614</v>
@@ -1403,16 +923,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>315.95</v>
+        <v>330.33</v>
       </c>
       <c r="C3" t="n">
-        <v>12.4</v>
+        <v>14.6</v>
       </c>
       <c r="D3" t="n">
-        <v>297.25</v>
+        <v>297.23</v>
       </c>
       <c r="E3" t="n">
-        <v>286.8</v>
+        <v>286.78</v>
       </c>
       <c r="F3" t="n">
         <v>0.258</v>
@@ -1439,16 +959,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>664.0599999999999</v>
+        <v>1720.07</v>
       </c>
       <c r="C4" t="n">
-        <v>103.56</v>
+        <v>494.1</v>
       </c>
       <c r="D4" t="n">
-        <v>40.65</v>
+        <v>40.67</v>
       </c>
       <c r="E4" t="n">
-        <v>37.65</v>
+        <v>37.61</v>
       </c>
       <c r="F4" t="n">
         <v>0.265</v>
@@ -1475,16 +995,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>677.8</v>
+        <v>1739.57</v>
       </c>
       <c r="C5" t="n">
-        <v>24.29</v>
+        <v>125.61</v>
       </c>
       <c r="D5" t="n">
-        <v>76.67</v>
+        <v>76.63</v>
       </c>
       <c r="E5" t="n">
-        <v>67.73999999999999</v>
+        <v>67.73</v>
       </c>
       <c r="F5" t="n">
         <v>0.666</v>
@@ -1511,16 +1031,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>220.33</v>
+        <v>220</v>
       </c>
       <c r="C6" t="n">
-        <v>89.81999999999999</v>
+        <v>117.15</v>
       </c>
       <c r="D6" t="n">
         <v>1212.83</v>
       </c>
       <c r="E6" t="n">
-        <v>1200.58</v>
+        <v>1200.59</v>
       </c>
       <c r="F6" t="n">
         <v>0.578</v>
@@ -1551,7 +1071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1562,42 +1082,47 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>HA_medio_mm_d</t>
+          <t>Par</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Mediana</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Desv_Est</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>n_pares</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>MATLAB_ref_mm_d</t>
+          <t>IQR</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Delta_pct</t>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Max</t>
         </is>
       </c>
     </row>
@@ -1607,153 +1132,718 @@
           <t>TC1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>337.3</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>sup→int</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>328</v>
+        <v>78</v>
       </c>
       <c r="D2" t="n">
-        <v>336.9</v>
+        <v>359.5</v>
       </c>
       <c r="E2" t="n">
-        <v>346.3</v>
+        <v>384.5</v>
       </c>
       <c r="F2" t="n">
-        <v>18.4</v>
+        <v>218.8</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>467.1</v>
       </c>
       <c r="H2" t="n">
-        <v>281</v>
+        <v>248.3</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>176.2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>634.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TC2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>315.9</v>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>int→inf</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>309.7</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>315.7</v>
+        <v>365.3</v>
       </c>
       <c r="E3" t="n">
-        <v>322.1</v>
+        <v>290</v>
       </c>
       <c r="F3" t="n">
-        <v>12.4</v>
+        <v>202.6</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>313.8</v>
       </c>
       <c r="H3" t="n">
-        <v>311</v>
+        <v>111.2</v>
       </c>
       <c r="I3" t="n">
-        <v>1.6</v>
+        <v>145.9</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1581.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>664.1</v>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sup→inf</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>608.3</v>
+        <v>76</v>
       </c>
       <c r="D4" t="n">
-        <v>645.7</v>
+        <v>415.1</v>
       </c>
       <c r="E4" t="n">
-        <v>710.6</v>
+        <v>276.7</v>
       </c>
       <c r="F4" t="n">
-        <v>103.6</v>
+        <v>243.3</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>627.7</v>
       </c>
       <c r="H4" t="n">
-        <v>2246</v>
+        <v>384.4</v>
       </c>
       <c r="I4" t="n">
-        <v>-70.40000000000001</v>
+        <v>183.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>945.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC4</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>677.8</v>
+          <t>TC1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>665.4</v>
+        <v>194</v>
       </c>
       <c r="D5" t="n">
-        <v>676.8</v>
+        <v>382.5</v>
       </c>
       <c r="E5" t="n">
-        <v>689.7</v>
+        <v>293.2</v>
       </c>
       <c r="F5" t="n">
-        <v>24.3</v>
+        <v>221.3</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>459.9</v>
       </c>
       <c r="H5" t="n">
-        <v>1555</v>
+        <v>238.5</v>
       </c>
       <c r="I5" t="n">
-        <v>-56.4</v>
+        <v>145.9</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1581.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D6" t="n">
+        <v>353</v>
+      </c>
+      <c r="E6" t="n">
+        <v>336.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>324.8</v>
+      </c>
+      <c r="G6" t="n">
+        <v>368.8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>44</v>
+      </c>
+      <c r="I6" t="n">
+        <v>266.9</v>
+      </c>
+      <c r="J6" t="n">
+        <v>461.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>21</v>
+      </c>
+      <c r="D7" t="n">
+        <v>348.6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>329.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>310.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>380.3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>285.2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>504.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>23</v>
+      </c>
+      <c r="D8" t="n">
+        <v>352.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>362.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>327.6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>370.8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>312.7</v>
+      </c>
+      <c r="J8" t="n">
+        <v>378.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>351.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>336.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>323.6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>372.4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>266.9</v>
+      </c>
+      <c r="J9" t="n">
+        <v>504.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1756.6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1988.9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1627.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2066.2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>438.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>421.3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2371.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>48</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3585.8</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2557.6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2107</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5737.4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3630.4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1303.6</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8627.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>52</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2136.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2255</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1990.3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2414</v>
+      </c>
+      <c r="H12" t="n">
+        <v>423.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>666</v>
+      </c>
+      <c r="J12" t="n">
+        <v>3323</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>150</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2473.6</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2190</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1848.1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2522.4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>674.3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>421.3</v>
+      </c>
+      <c r="J13" t="n">
+        <v>8627.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>103</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1780.1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1846.4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1449.4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2087.4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>638</v>
+      </c>
+      <c r="I14" t="n">
+        <v>603.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2697.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>95</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2410.6</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2531.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1205.9</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3314.2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2108.3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>755.5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4117</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>99</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1974.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2183.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1305.4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2472.9</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1167.5</v>
+      </c>
+      <c r="I16" t="n">
+        <v>736.7</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2914.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TC4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>297</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2046.5</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2032.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1356.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2497.6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1141</v>
+      </c>
+      <c r="I17" t="n">
+        <v>603.1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4117</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>TC5</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>220.3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>173.4</v>
-      </c>
-      <c r="D6" t="n">
-        <v>211.8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>262.9</v>
-      </c>
-      <c r="F6" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" t="n">
-        <v>181</v>
-      </c>
-      <c r="I6" t="n">
-        <v>21.7</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sup→int</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>93</v>
+      </c>
+      <c r="D18" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>107</v>
+      </c>
+      <c r="G18" t="n">
+        <v>129.3</v>
+      </c>
+      <c r="H18" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="I18" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="J18" t="n">
+        <v>168.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>int→inf</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>57</v>
+      </c>
+      <c r="D19" t="n">
+        <v>344.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>319.4</v>
+      </c>
+      <c r="F19" t="n">
+        <v>242.2</v>
+      </c>
+      <c r="G19" t="n">
+        <v>411</v>
+      </c>
+      <c r="H19" t="n">
+        <v>168.8</v>
+      </c>
+      <c r="I19" t="n">
+        <v>170.2</v>
+      </c>
+      <c r="J19" t="n">
+        <v>927.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>sup→inf</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>59</v>
+      </c>
+      <c r="D20" t="n">
+        <v>200.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>190.9</v>
+      </c>
+      <c r="F20" t="n">
+        <v>164.7</v>
+      </c>
+      <c r="G20" t="n">
+        <v>226.7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>62</v>
+      </c>
+      <c r="I20" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J20" t="n">
+        <v>329.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TC5</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>209</v>
+      </c>
+      <c r="D21" t="n">
+        <v>203.3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>163.8</v>
+      </c>
+      <c r="F21" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="G21" t="n">
+        <v>240.6</v>
+      </c>
+      <c r="H21" t="n">
+        <v>123.8</v>
+      </c>
+      <c r="I21" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>927.8</v>
       </c>
     </row>
   </sheetData>
@@ -1834,7 +1924,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.795</v>
+        <v>0.798</v>
       </c>
       <c r="D2" t="n">
         <v>0.728</v>
@@ -1843,7 +1933,7 @@
         <v>0.483</v>
       </c>
       <c r="F2" t="n">
-        <v>0.864</v>
+        <v>0.878</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -1852,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>319.1</v>
+        <v>314.1</v>
       </c>
       <c r="J2" t="n">
         <v>275.7</v>
@@ -1870,7 +1960,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.577</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="D3" t="n">
         <v>0.483</v>
@@ -1879,7 +1969,7 @@
         <v>0.103</v>
       </c>
       <c r="F3" t="n">
-        <v>0.543</v>
+        <v>0.506</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -1888,7 +1978,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>355.8</v>
+        <v>381.9</v>
       </c>
       <c r="J3" t="n">
         <v>193.1</v>
@@ -1906,7 +1996,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.588</v>
+        <v>0.59</v>
       </c>
       <c r="D4" t="n">
         <v>0.728</v>
@@ -1915,7 +2005,7 @@
         <v>0.103</v>
       </c>
       <c r="F4" t="n">
-        <v>0.342</v>
+        <v>0.351</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -1924,7 +2014,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>336.9</v>
+        <v>345.9</v>
       </c>
       <c r="J4" t="n">
         <v>984.7</v>
@@ -1942,7 +2032,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.594</v>
+        <v>0.589</v>
       </c>
       <c r="D5" t="n">
         <v>0.619</v>
@@ -1951,7 +2041,7 @@
         <v>0.218</v>
       </c>
       <c r="F5" t="n">
-        <v>0.382</v>
+        <v>0.364</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -1960,7 +2050,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>328.5</v>
+        <v>345.1</v>
       </c>
       <c r="J5" t="n">
         <v>125.4</v>
@@ -1978,7 +2068,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.472</v>
+        <v>0.468</v>
       </c>
       <c r="D6" t="n">
         <v>0.218</v>
@@ -1987,7 +2077,7 @@
         <v>0.022</v>
       </c>
       <c r="F6" t="n">
-        <v>0.454</v>
+        <v>0.437</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -1996,7 +2086,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>303.7</v>
+        <v>315.9</v>
       </c>
       <c r="J6" t="n">
         <v>138</v>
@@ -2014,7 +2104,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.585</v>
+        <v>0.59</v>
       </c>
       <c r="D7" t="n">
         <v>0.619</v>
@@ -2023,7 +2113,7 @@
         <v>0.022</v>
       </c>
       <c r="F7" t="n">
-        <v>0.502</v>
+        <v>0.525</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -2032,7 +2122,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>315.7</v>
+        <v>330</v>
       </c>
       <c r="J7" t="n">
         <v>628.3</v>
@@ -2050,7 +2140,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.61</v>
+        <v>0.528</v>
       </c>
       <c r="D8" t="n">
         <v>0.606</v>
@@ -2059,16 +2149,16 @@
         <v>0.73</v>
       </c>
       <c r="F8" t="n">
-        <v>0.049</v>
+        <v>0.022</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>570.9</v>
+        <v>1281.9</v>
       </c>
       <c r="J8" t="n">
         <v>27.9</v>
@@ -2086,7 +2176,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.581</v>
+        <v>0.487</v>
       </c>
       <c r="D9" t="n">
         <v>0.73</v>
@@ -2095,16 +2185,16 @@
         <v>0.6919999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>0.014</v>
+        <v>0.005</v>
       </c>
       <c r="G9" t="n">
-        <v>0.707</v>
+        <v>0.1</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>775.6</v>
+        <v>2255.6</v>
       </c>
       <c r="J9" t="n">
         <v>11.1</v>
@@ -2122,7 +2212,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.611</v>
+        <v>0.528</v>
       </c>
       <c r="D10" t="n">
         <v>0.606</v>
@@ -2131,16 +2221,16 @@
         <v>0.6919999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>0.129</v>
+        <v>0.051</v>
       </c>
       <c r="G10" t="n">
-        <v>0.924</v>
+        <v>0.5</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>645.7</v>
+        <v>1622.7</v>
       </c>
       <c r="J10" t="n">
         <v>83</v>
@@ -2158,7 +2248,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.668</v>
+        <v>0.597</v>
       </c>
       <c r="D11" t="n">
         <v>0.836</v>
@@ -2167,16 +2257,16 @@
         <v>0.782</v>
       </c>
       <c r="F11" t="n">
-        <v>0.064</v>
+        <v>0.026</v>
       </c>
       <c r="G11" t="n">
-        <v>0.91</v>
+        <v>0.5</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>654</v>
+        <v>1617.1</v>
       </c>
       <c r="J11" t="n">
         <v>41.7</v>
@@ -2194,7 +2284,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.632</v>
+        <v>0.575</v>
       </c>
       <c r="D12" t="n">
         <v>0.782</v>
@@ -2203,16 +2293,16 @@
         <v>0.75</v>
       </c>
       <c r="F12" t="n">
-        <v>0.048</v>
+        <v>0.018</v>
       </c>
       <c r="G12" t="n">
-        <v>0.829</v>
+        <v>0.5</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>702.6</v>
+        <v>1868.1</v>
       </c>
       <c r="J12" t="n">
         <v>33.5</v>
@@ -2230,7 +2320,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.697</v>
+        <v>0.606</v>
       </c>
       <c r="D13" t="n">
         <v>0.836</v>
@@ -2239,16 +2329,16 @@
         <v>0.75</v>
       </c>
       <c r="F13" t="n">
-        <v>0.229</v>
+        <v>0.089</v>
       </c>
       <c r="G13" t="n">
-        <v>0.872</v>
+        <v>0.5</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>676.8</v>
+        <v>1733.5</v>
       </c>
       <c r="J13" t="n">
         <v>154.7</v>
@@ -2266,7 +2356,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.577</v>
+        <v>0.569</v>
       </c>
       <c r="D14" t="n">
         <v>0.8129999999999999</v>
@@ -2275,7 +2365,7 @@
         <v>0.128</v>
       </c>
       <c r="F14" t="n">
-        <v>0.192</v>
+        <v>0.162</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -2284,7 +2374,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>135.1</v>
+        <v>113.7</v>
       </c>
       <c r="J14" t="n">
         <v>703</v>
@@ -2302,7 +2392,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.582</v>
       </c>
       <c r="D15" t="n">
         <v>0.128</v>
@@ -2311,7 +2401,7 @@
         <v>0.023</v>
       </c>
       <c r="F15" t="n">
-        <v>0.894</v>
+        <v>0.984</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -2320,7 +2410,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>314.1</v>
+        <v>345.6</v>
       </c>
       <c r="J15" t="n">
         <v>351.3</v>
@@ -2338,7 +2428,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.528</v>
+        <v>0.527</v>
       </c>
       <c r="D16" t="n">
         <v>0.8129999999999999</v>
@@ -2347,7 +2437,7 @@
         <v>0.023</v>
       </c>
       <c r="F16" t="n">
-        <v>0.082</v>
+        <v>0.078</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
@@ -2356,7 +2446,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>211.8</v>
+        <v>200.7</v>
       </c>
       <c r="J16" t="n">
         <v>2584.2</v>
@@ -2430,19 +2520,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>319.1</v>
+        <v>314.1</v>
       </c>
       <c r="D2" t="n">
         <v>12.9</v>
       </c>
       <c r="E2" t="n">
-        <v>41.3</v>
+        <v>40.6</v>
       </c>
       <c r="F2" t="n">
-        <v>238.2</v>
+        <v>234.5</v>
       </c>
       <c r="G2" t="n">
-        <v>400</v>
+        <v>393.6</v>
       </c>
       <c r="H2" t="n">
         <v>10</v>
@@ -2460,19 +2550,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>355.8</v>
+        <v>381.9</v>
       </c>
       <c r="D3" t="n">
         <v>21.6</v>
       </c>
       <c r="E3" t="n">
-        <v>76.90000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>205.1</v>
+        <v>220.1</v>
       </c>
       <c r="G3" t="n">
-        <v>506.6</v>
+        <v>543.7</v>
       </c>
       <c r="H3" t="n">
         <v>20</v>
@@ -2490,19 +2580,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>336.9</v>
+        <v>345.9</v>
       </c>
       <c r="D4" t="n">
         <v>21.6</v>
       </c>
       <c r="E4" t="n">
-        <v>72.8</v>
+        <v>74.8</v>
       </c>
       <c r="F4" t="n">
-        <v>194.2</v>
+        <v>199.3</v>
       </c>
       <c r="G4" t="n">
-        <v>479.6</v>
+        <v>492.4</v>
       </c>
       <c r="H4" t="n">
         <v>20</v>
@@ -2520,19 +2610,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>328.5</v>
+        <v>345.1</v>
       </c>
       <c r="D5" t="n">
         <v>21.6</v>
       </c>
       <c r="E5" t="n">
-        <v>71</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>189.3</v>
+        <v>198.9</v>
       </c>
       <c r="G5" t="n">
-        <v>467.6</v>
+        <v>491.2</v>
       </c>
       <c r="H5" t="n">
         <v>20</v>
@@ -2550,19 +2640,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>303.7</v>
+        <v>315.9</v>
       </c>
       <c r="D6" t="n">
         <v>21.6</v>
       </c>
       <c r="E6" t="n">
-        <v>65.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="F6" t="n">
-        <v>175</v>
+        <v>182.1</v>
       </c>
       <c r="G6" t="n">
-        <v>432.3</v>
+        <v>449.8</v>
       </c>
       <c r="H6" t="n">
         <v>20</v>
@@ -2580,19 +2670,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>315.7</v>
+        <v>330</v>
       </c>
       <c r="D7" t="n">
         <v>21.6</v>
       </c>
       <c r="E7" t="n">
-        <v>68.2</v>
+        <v>71.3</v>
       </c>
       <c r="F7" t="n">
-        <v>182</v>
+        <v>190.2</v>
       </c>
       <c r="G7" t="n">
-        <v>449.4</v>
+        <v>469.8</v>
       </c>
       <c r="H7" t="n">
         <v>20</v>
@@ -2610,19 +2700,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>570.9</v>
+        <v>1281.9</v>
       </c>
       <c r="D8" t="n">
         <v>12.9</v>
       </c>
       <c r="E8" t="n">
-        <v>73.8</v>
+        <v>165.7</v>
       </c>
       <c r="F8" t="n">
-        <v>426.2</v>
+        <v>957</v>
       </c>
       <c r="G8" t="n">
-        <v>715.6</v>
+        <v>1606.7</v>
       </c>
       <c r="H8" t="n">
         <v>10</v>
@@ -2640,19 +2730,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>775.6</v>
+        <v>2255.6</v>
       </c>
       <c r="D9" t="n">
         <v>12.9</v>
       </c>
       <c r="E9" t="n">
-        <v>100.3</v>
+        <v>291.7</v>
       </c>
       <c r="F9" t="n">
-        <v>579</v>
+        <v>1684</v>
       </c>
       <c r="G9" t="n">
-        <v>972.1</v>
+        <v>2827.3</v>
       </c>
       <c r="H9" t="n">
         <v>10</v>
@@ -2670,19 +2760,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>645.7</v>
+        <v>1622.7</v>
       </c>
       <c r="D10" t="n">
         <v>12.9</v>
       </c>
       <c r="E10" t="n">
-        <v>83.5</v>
+        <v>209.8</v>
       </c>
       <c r="F10" t="n">
-        <v>482.1</v>
+        <v>1211.5</v>
       </c>
       <c r="G10" t="n">
-        <v>809.3</v>
+        <v>2034</v>
       </c>
       <c r="H10" t="n">
         <v>10</v>
@@ -2700,19 +2790,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>654</v>
+        <v>1617.1</v>
       </c>
       <c r="D11" t="n">
         <v>9.6</v>
       </c>
       <c r="E11" t="n">
-        <v>62.8</v>
+        <v>155.3</v>
       </c>
       <c r="F11" t="n">
-        <v>531</v>
+        <v>1312.8</v>
       </c>
       <c r="G11" t="n">
-        <v>777.1</v>
+        <v>1921.4</v>
       </c>
       <c r="H11" t="n">
         <v>5</v>
@@ -2730,19 +2820,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>702.6</v>
+        <v>1868.1</v>
       </c>
       <c r="D12" t="n">
         <v>12.9</v>
       </c>
       <c r="E12" t="n">
-        <v>90.8</v>
+        <v>241.5</v>
       </c>
       <c r="F12" t="n">
-        <v>524.5</v>
+        <v>1394.6</v>
       </c>
       <c r="G12" t="n">
-        <v>880.6</v>
+        <v>2341.5</v>
       </c>
       <c r="H12" t="n">
         <v>10</v>
@@ -2760,19 +2850,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>676.8</v>
+        <v>1733.5</v>
       </c>
       <c r="D13" t="n">
         <v>12.9</v>
       </c>
       <c r="E13" t="n">
-        <v>87.5</v>
+        <v>224.1</v>
       </c>
       <c r="F13" t="n">
-        <v>505.3</v>
+        <v>1294.1</v>
       </c>
       <c r="G13" t="n">
-        <v>848.3</v>
+        <v>2172.8</v>
       </c>
       <c r="H13" t="n">
         <v>10</v>
@@ -2790,19 +2880,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>135.1</v>
+        <v>113.7</v>
       </c>
       <c r="D14" t="n">
         <v>21.6</v>
       </c>
       <c r="E14" t="n">
-        <v>29.2</v>
+        <v>24.6</v>
       </c>
       <c r="F14" t="n">
-        <v>77.90000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="G14" t="n">
-        <v>192.3</v>
+        <v>161.9</v>
       </c>
       <c r="H14" t="n">
         <v>20</v>
@@ -2820,19 +2910,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>314.1</v>
+        <v>345.6</v>
       </c>
       <c r="D15" t="n">
         <v>21.6</v>
       </c>
       <c r="E15" t="n">
-        <v>67.90000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="F15" t="n">
-        <v>181</v>
+        <v>199.2</v>
       </c>
       <c r="G15" t="n">
-        <v>447.2</v>
+        <v>492.1</v>
       </c>
       <c r="H15" t="n">
         <v>20</v>
@@ -2850,19 +2940,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>211.8</v>
+        <v>200.7</v>
       </c>
       <c r="D16" t="n">
         <v>21.6</v>
       </c>
       <c r="E16" t="n">
-        <v>45.8</v>
+        <v>43.4</v>
       </c>
       <c r="F16" t="n">
-        <v>122.1</v>
+        <v>115.7</v>
       </c>
       <c r="G16" t="n">
-        <v>301.5</v>
+        <v>285.8</v>
       </c>
       <c r="H16" t="n">
         <v>20</v>
@@ -2879,7 +2969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2910,22 +3000,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>fase_deg</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>offset_C</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>n_dias_ajuste</t>
+          <t>n_dias</t>
         </is>
       </c>
     </row>
@@ -2950,15 +3030,9 @@
         <v>1.5242</v>
       </c>
       <c r="F2" t="n">
-        <v>87.3</v>
+        <v>0.728</v>
       </c>
       <c r="G2" t="n">
-        <v>18.28</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.728</v>
-      </c>
-      <c r="I2" t="n">
         <v>65</v>
       </c>
     </row>
@@ -2983,15 +3057,9 @@
         <v>0.1391</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>0.483</v>
       </c>
       <c r="G3" t="n">
-        <v>17.49</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.483</v>
-      </c>
-      <c r="I3" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3016,15 +3084,9 @@
         <v>6.2051</v>
       </c>
       <c r="F4" t="n">
-        <v>355.5</v>
+        <v>0.1028</v>
       </c>
       <c r="G4" t="n">
-        <v>17.57</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1028</v>
-      </c>
-      <c r="I4" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3049,15 +3111,9 @@
         <v>0.3039</v>
       </c>
       <c r="F5" t="n">
-        <v>17.4</v>
+        <v>0.6192</v>
       </c>
       <c r="G5" t="n">
-        <v>17.01</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.6192</v>
-      </c>
-      <c r="I5" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3082,15 +3138,9 @@
         <v>4.9513</v>
       </c>
       <c r="F6" t="n">
-        <v>283.7</v>
+        <v>0.218</v>
       </c>
       <c r="G6" t="n">
-        <v>17.15</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.218</v>
-      </c>
-      <c r="I6" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3115,15 +3165,9 @@
         <v>3.4749</v>
       </c>
       <c r="F7" t="n">
-        <v>199.1</v>
+        <v>0.0216</v>
       </c>
       <c r="G7" t="n">
-        <v>17.3</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0216</v>
-      </c>
-      <c r="I7" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3148,15 +3192,9 @@
         <v>0.4528</v>
       </c>
       <c r="F8" t="n">
-        <v>25.9</v>
+        <v>0.6062</v>
       </c>
       <c r="G8" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.6062</v>
-      </c>
-      <c r="I8" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3181,15 +3219,9 @@
         <v>6.1382</v>
       </c>
       <c r="F9" t="n">
-        <v>351.7</v>
+        <v>0.7295</v>
       </c>
       <c r="G9" t="n">
-        <v>18.07</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.7295</v>
-      </c>
-      <c r="I9" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3214,15 +3246,9 @@
         <v>5.8559</v>
       </c>
       <c r="F10" t="n">
-        <v>335.5</v>
+        <v>0.6924</v>
       </c>
       <c r="G10" t="n">
-        <v>18.09</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.6924</v>
-      </c>
-      <c r="I10" t="n">
         <v>32</v>
       </c>
     </row>
@@ -3247,15 +3273,9 @@
         <v>1.2132</v>
       </c>
       <c r="F11" t="n">
-        <v>69.5</v>
+        <v>0.8363</v>
       </c>
       <c r="G11" t="n">
-        <v>18.49</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.8363</v>
-      </c>
-      <c r="I11" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3280,15 +3300,9 @@
         <v>0.978</v>
       </c>
       <c r="F12" t="n">
-        <v>56</v>
+        <v>0.7824</v>
       </c>
       <c r="G12" t="n">
-        <v>18.25</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.7824</v>
-      </c>
-      <c r="I12" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3313,15 +3327,9 @@
         <v>0.8567</v>
       </c>
       <c r="F13" t="n">
-        <v>49.1</v>
+        <v>0.7496</v>
       </c>
       <c r="G13" t="n">
-        <v>18.31</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.7496</v>
-      </c>
-      <c r="I13" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3346,15 +3354,9 @@
         <v>1.0866</v>
       </c>
       <c r="F14" t="n">
-        <v>62.3</v>
+        <v>0.8128</v>
       </c>
       <c r="G14" t="n">
-        <v>18.23</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.8128</v>
-      </c>
-      <c r="I14" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3379,15 +3381,9 @@
         <v>4.8139</v>
       </c>
       <c r="F15" t="n">
-        <v>275.8</v>
+        <v>0.1276</v>
       </c>
       <c r="G15" t="n">
-        <v>18.33</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.1276</v>
-      </c>
-      <c r="I15" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3412,15 +3408,9 @@
         <v>2.1943</v>
       </c>
       <c r="F16" t="n">
-        <v>125.7</v>
+        <v>0.0225</v>
       </c>
       <c r="G16" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="I16" t="n">
         <v>65</v>
       </c>
     </row>
@@ -3435,7 +3425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3479,11 +3469,6 @@
           <t>USCS</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>fuente</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3514,11 +3499,6 @@
           <t>SP-SM</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>IDIEM OT-10 Feb-Mar 2026</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3549,11 +3529,6 @@
           <t>SM</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>IDIEM OT-10 Feb-Mar 2026</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3584,11 +3559,6 @@
           <t>SW-SM</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>IDIEM OT-10 Feb-Mar 2026</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3619,11 +3589,6 @@
           <t>GP-GM</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>IDIEM OT-10 Feb-Mar 2026</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3652,11 +3617,6 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>SW-SM</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>IDIEM OT-10 Feb-Mar 2026</t>
         </is>
       </c>
     </row>

</xml_diff>